<commit_message>
optimized speed of beta computation
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>8.85%</t>
+          <t>20.41%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>6.88%</t>
+          <t>15.88%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>8.78%</t>
+          <t>19.90%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>6.17%</t>
+          <t>11.76%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>9.02%</t>
+          <t>20.82%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>13.31%</t>
+          <t>30.71%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-20.54%</t>
+          <t>-42.10%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-41.99%</t>
+          <t>-73.54%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.22</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-7.29%</t>
+          <t>-16.82%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-20.12%</t>
+          <t>-46.43%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[6.32%, 11.37%]</t>
+          <t>[14.58%, 26.25%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[3.15%, 10.61%]</t>
+          <t>[7.27%, 24.49%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>5.18%</t>
+          <t>17.46%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>3.21%</t>
+          <t>12.92%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>1.43%</t>
+          <t>3.24%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.21%</t>
+          <t>4.99%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>3.63</t>
+          <t>5.38</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.1454</t>
+          <t>0.0096</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[2.38%, 7.98%]</t>
+          <t>[11.10%, 23.82%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[-1.11%, 7.54%]</t>
+          <t>[3.14%, 22.70%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.061</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.061</t>
+          <t>-0.146</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-2.32</t>
+          <t>-2.41</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-1.03</t>
+          <t>-1.07</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">

</xml_diff>

<commit_message>
adjusted output and optimization
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>20.41%</t>
+          <t>10.21%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>15.88%</t>
+          <t>7.94%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>19.90%</t>
+          <t>10.11%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>6.98%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>20.82%</t>
+          <t>10.41%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>30.71%</t>
+          <t>15.36%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-42.10%</t>
+          <t>-23.37%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-73.54%</t>
+          <t>-46.87%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.48</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.22</t>
+          <t>0.17</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-16.82%</t>
+          <t>-8.41%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-46.43%</t>
+          <t>-23.22%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[14.58%, 26.25%]</t>
+          <t>[7.29%, 13.12%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[7.27%, 24.49%]</t>
+          <t>[3.64%, 12.24%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>17.46%</t>
+          <t>6.62%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>12.92%</t>
+          <t>4.36%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>3.24%</t>
+          <t>1.64%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>4.99%</t>
+          <t>2.53%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>5.38</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>0.0000</t>
+          <t>0.0001</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0096</t>
+          <t>0.0854</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[11.10%, 23.82%]</t>
+          <t>[3.41%, 9.84%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[3.14%, 22.70%]</t>
+          <t>[-0.61%, 9.32%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.146</t>
+          <t>-0.071</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.146</t>
+          <t>-0.071</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-2.41</t>
+          <t>-2.34</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-1.07</t>
+          <t>-1.04</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Added failure model factors to short book
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>11.84%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>7.94%</t>
+          <t>8.27%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>-10.43%</t>
+          <t>-10.10%</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>-9.76%</t>
+          <t>-10.42%</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>11.89%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>6.98%</t>
+          <t>7.17%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>-11.98%</t>
+          <t>-12.15%</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>-11.02%</t>
+          <t>-12.13%</t>
         </is>
       </c>
     </row>
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>10.40%</t>
+          <t>10.59%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>16.21%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>21.37%</t>
+          <t>23.65%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>19.32%</t>
+          <t>22.14%</t>
         </is>
       </c>
     </row>
@@ -865,12 +865,12 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.51</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>-0.49</t>
+          <t>-0.43</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>-0.51</t>
+          <t>-0.47</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-23.36%</t>
+          <t>-22.69%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-46.82%</t>
+          <t>-41.34%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>-99.82%</t>
+          <t>-99.84%</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="G13" s="22" t="inlineStr">
         <is>
-          <t>-99.68%</t>
+          <t>-99.84%</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>-0.66</t>
+          <t>-0.58</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>-0.67</t>
+          <t>-0.63</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>0.52</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-8.40%</t>
+          <t>-10.13%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-23.21%</t>
+          <t>-25.57%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>-26.81%</t>
+          <t>-30.22%</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>-25.01%</t>
+          <t>-28.42%</t>
         </is>
       </c>
     </row>
@@ -1057,32 +1057,32 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
+          <t>62.4%</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>55.5%</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>63.0%</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>42.4%</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
           <t>61.7%</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>55.7%</t>
-        </is>
-      </c>
-      <c r="D18" s="18" t="inlineStr">
-        <is>
-          <t>63.0%</t>
-        </is>
-      </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="G18" s="19" t="inlineStr">
         <is>
           <t>40.5%</t>
-        </is>
-      </c>
-      <c r="F18" s="18" t="inlineStr">
-        <is>
-          <t>61.7%</t>
-        </is>
-      </c>
-      <c r="G18" s="19" t="inlineStr">
-        <is>
-          <t>40.2%</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>0.12</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>-0.16</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>0.59</t>
+          <t>0.44</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>0.46</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>0.92</t>
+          <t>0.68</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>2.84</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>2.65</t>
+          <t>2.42</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>2.62</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>6.86</t>
+          <t>7.82</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>3.57</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>-3.41</t>
+          <t>-2.99</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>-3.53</t>
+          <t>-3.29</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.0004</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>0.0007</t>
+          <t>0.0029</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>0.0004</t>
+          <t>0.0010</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[7.29%, 13.12%]</t>
+          <t>[8.87%, 14.81%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[3.63%, 12.24%]</t>
+          <t>[3.72%, 12.81%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>[-16.42%, -4.44%]</t>
+          <t>[-16.72%, -3.47%]</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>[-15.17%, -4.35%]</t>
+          <t>[-16.63%, -4.22%]</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>8.77%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>5.43%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>0.17%</t>
+          <t>1.63%</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>-0.16%</t>
+          <t>0.46%</t>
         </is>
       </c>
     </row>
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.72%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.26%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>1.27%</t>
+          <t>1.46%</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>1.24%</t>
+          <t>1.29%</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>5.09</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>0.36</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0855</t>
+          <t>0.0165</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>0.8942</t>
+          <t>0.2622</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>0.8961</t>
+          <t>0.7223</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[3.41%, 9.83%]</t>
+          <t>[5.40%, 12.15%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[-0.61%, 9.31%]</t>
+          <t>[0.99%, 9.86%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>[-2.32%, 2.66%]</t>
+          <t>[-1.22%, 4.49%]</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[-2.59%, 2.27%]</t>
+          <t>[-2.06%, 2.98%]</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.071</t>
+          <t>-0.133</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.071</t>
+          <t>-0.161</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-1.274</t>
+          <t>-1.410</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>-1.154</t>
+          <t>-1.308</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-2.35</t>
+          <t>-4.23</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-1.04</t>
+          <t>-2.43</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>-39.62</t>
+          <t>-35.74</t>
         </is>
       </c>
       <c r="F32" s="21" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>-34.65</t>
+          <t>-31.18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update output files for failure-model branch
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -628,7 +628,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Composite z-score: Shareholder Yield + Gross Profitability + ROIC  |  130% long top-100 / w_short = 130% × β_long/β_short (Vasicek-adj, 12m trailing)  |  Monthly rebalancing, ±5 pp sector neutrality, beta-neutral</t>
+          <t>Composite z-score: Shareholder Yield + Gross Profitability + ROIC  |  175% long top-100 / w_short = 175% × β_long/β_short (Vasicek-adj, 12m trailing)  |  Monthly rebalancing, ±5% sector neutrality, beta-neutral</t>
         </is>
       </c>
     </row>
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>11.84%</t>
+          <t>13.81%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>8.27%</t>
+          <t>9.64%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>11.89%</t>
+          <t>13.87%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>7.17%</t>
+          <t>8.13%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>10.59%</t>
+          <t>12.36%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>16.21%</t>
+          <t>18.91%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-22.69%</t>
+          <t>-26.05%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-41.34%</t>
+          <t>-46.58%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.53</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.21</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-10.13%</t>
+          <t>-11.81%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-25.57%</t>
+          <t>-29.84%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[8.87%, 14.81%]</t>
+          <t>[10.35%, 17.27%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[3.72%, 12.81%]</t>
+          <t>[4.34%, 14.94%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>8.77%</t>
+          <t>10.94%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>5.43%</t>
+          <t>7.03%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>1.72%</t>
+          <t>2.00%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.26%</t>
+          <t>2.63%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>5.09</t>
+          <t>5.46</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>2.68</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0165</t>
+          <t>0.0075</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[5.40%, 12.15%]</t>
+          <t>[7.01%, 14.86%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[0.99%, 9.86%]</t>
+          <t>[1.88%, 12.18%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.133</t>
+          <t>-0.156</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.161</t>
+          <t>-0.188</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-4.23</t>
+          <t>-4.24</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-2.43</t>
+          <t>-2.44</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Update LONG_WEIGHT to 1.75, import constants in make_table/make_plots/export_holdings
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -628,7 +628,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Composite z-score: Shareholder Yield + Gross Profitability + ROIC  |  130% long top-100 / w_short = 130% × β_long/β_short (Vasicek-adj, 12m trailing)  |  Monthly rebalancing, ±5 pp sector neutrality, beta-neutral</t>
+          <t>Composite z-score: Shareholder Yield + Gross Profitability + ROIC  |  175% long top-100 / w_short = 175% × β_long/β_short (Vasicek-adj, 12m trailing)  |  Monthly rebalancing, ±5% sector neutrality, beta-neutral</t>
         </is>
       </c>
     </row>
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>11.90%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>7.94%</t>
+          <t>9.26%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>10.11%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>6.98%</t>
+          <t>7.94%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>10.40%</t>
+          <t>12.14%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>15.35%</t>
+          <t>17.91%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-23.36%</t>
+          <t>-26.78%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-46.82%</t>
+          <t>-52.43%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.17</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-8.40%</t>
+          <t>-9.80%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-23.21%</t>
+          <t>-27.08%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[7.29%, 13.12%]</t>
+          <t>[8.50%, 15.31%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[3.63%, 12.24%]</t>
+          <t>[4.24%, 14.28%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>6.62%</t>
+          <t>8.43%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>4.35%</t>
+          <t>5.78%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>1.64%</t>
+          <t>1.90%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.53%</t>
+          <t>2.94%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>4.43</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.97</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>0.0001</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0855</t>
+          <t>0.0492</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[3.41%, 9.83%]</t>
+          <t>[4.70%, 12.16%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[-0.61%, 9.31%]</t>
+          <t>[0.02%, 11.54%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.071</t>
+          <t>-0.084</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.071</t>
+          <t>-0.084</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-2.35</t>
+          <t>-2.37</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-1.04</t>
+          <t>-1.05</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Remove momentum and volatility from short signal, keep fundamental failure factors only
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>13.81%</t>
+          <t>11.46%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>9.64%</t>
+          <t>8.91%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>-10.10%</t>
+          <t>-10.32%</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>-10.42%</t>
+          <t>-9.63%</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>13.87%</t>
+          <t>11.35%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>8.13%</t>
+          <t>7.69%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>-12.15%</t>
+          <t>-11.84%</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>-12.13%</t>
+          <t>-10.92%</t>
         </is>
       </c>
     </row>
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>12.36%</t>
+          <t>11.58%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>18.91%</t>
+          <t>17.25%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>23.65%</t>
+          <t>21.16%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>22.14%</t>
+          <t>19.51%</t>
         </is>
       </c>
     </row>
@@ -865,12 +865,12 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>0.51</t>
+          <t>0.52</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
@@ -880,7 +880,7 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>-0.43</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>-0.47</t>
+          <t>-0.49</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-26.05%</t>
+          <t>-29.06%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-46.58%</t>
+          <t>-45.70%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>-99.84%</t>
+          <t>-99.81%</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="G13" s="22" t="inlineStr">
         <is>
-          <t>-99.84%</t>
+          <t>-99.70%</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>2.12</t>
+          <t>1.84</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>-0.58</t>
+          <t>-0.66</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>-0.63</t>
+          <t>-0.67</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>0.39</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.21</t>
+          <t>0.19</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-11.81%</t>
+          <t>-7.85%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-29.84%</t>
+          <t>-23.98%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>-30.22%</t>
+          <t>-20.68%</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>-28.42%</t>
+          <t>-20.20%</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1057,12 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>62.4%</t>
+          <t>61.8%</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>55.5%</t>
+          <t>56.4%</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>42.4%</t>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>40.5%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>-0.16</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>0.44</t>
+          <t>0.64</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>0.46</t>
+          <t>0.67</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>3.51</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>2.42</t>
+          <t>2.17</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>2.62</t>
+          <t>2.25</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>7.82</t>
+          <t>6.92</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>3.61</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>-2.99</t>
+          <t>-3.41</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>-3.29</t>
+          <t>-3.45</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>0.0004</t>
+          <t>0.0003</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>0.0029</t>
+          <t>0.0007</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>0.0010</t>
+          <t>0.0006</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[10.35%, 17.27%]</t>
+          <t>[8.21%, 14.70%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[4.34%, 14.94%]</t>
+          <t>[4.07%, 13.74%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>[-16.72%, -3.47%]</t>
+          <t>[-16.25%, -4.39%]</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>[-16.63%, -4.22%]</t>
+          <t>[-15.09%, -4.16%]</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>10.94%</t>
+          <t>8.09%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>7.03%</t>
+          <t>5.89%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>1.63%</t>
+          <t>0.28%</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>0.46%</t>
+          <t>0.22%</t>
         </is>
       </c>
     </row>
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>2.00%</t>
+          <t>1.92%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.63%</t>
+          <t>2.58%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>1.46%</t>
+          <t>1.22%</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>1.29%</t>
+          <t>1.03%</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>5.46</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2.68</t>
+          <t>2.28</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>0.36</t>
+          <t>0.21</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0075</t>
+          <t>0.0227</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>0.2622</t>
+          <t>0.8184</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>0.7223</t>
+          <t>0.8333</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[7.01%, 14.86%]</t>
+          <t>[4.33%, 11.86%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[1.88%, 12.18%]</t>
+          <t>[0.82%, 10.95%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>[-1.22%, 4.49%]</t>
+          <t>[-2.11%, 2.66%]</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[-2.06%, 2.98%]</t>
+          <t>[-1.80%, 2.24%]</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.156</t>
+          <t>-0.097</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.188</t>
+          <t>-0.139</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-1.410</t>
+          <t>-1.274</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>-1.308</t>
+          <t>-1.183</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-4.24</t>
+          <t>-2.97</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-2.44</t>
+          <t>-2.09</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>-35.74</t>
+          <t>-45.54</t>
         </is>
       </c>
       <c r="F32" s="21" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>-31.18</t>
+          <t>-47.85</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add TARGET_BETA=0.30 for net long bias instead of market neutral
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>11.46%</t>
+          <t>14.29%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>8.91%</t>
+          <t>11.55%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>11.35%</t>
+          <t>14.59%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>7.69%</t>
+          <t>10.75%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>11.58%</t>
+          <t>11.05%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>17.25%</t>
+          <t>16.17%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -865,12 +865,12 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>0.52</t>
+          <t>0.71</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-29.06%</t>
+          <t>-23.29%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-45.70%</t>
+          <t>-39.99%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>2.61</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>0.61</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>0.29</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-7.85%</t>
+          <t>-8.68%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-23.98%</t>
+          <t>-19.04%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>61.8%</t>
+          <t>65.2%</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>56.4%</t>
+          <t>57.9%</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>2.33</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>6.92</t>
+          <t>9.04</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>3.61</t>
+          <t>4.99</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>0.0003</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[8.21%, 14.70%]</t>
+          <t>[11.20%, 17.39%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[4.07%, 13.74%]</t>
+          <t>[7.02%, 16.08%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>8.09%</t>
+          <t>8.27%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>5.89%</t>
+          <t>6.04%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>1.92%</t>
+          <t>1.75%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.58%</t>
+          <t>2.42%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>4.22</t>
+          <t>4.71</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2.28</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0227</t>
+          <t>0.0124</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[4.33%, 11.86%]</t>
+          <t>[4.83%, 11.71%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[0.82%, 10.95%]</t>
+          <t>[1.30%, 10.78%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>-0.097</t>
+          <t>0.222</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>-0.139</t>
+          <t>0.160</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>-2.97</t>
+          <t>7.43</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>-2.09</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">

</xml_diff>

<commit_message>
final adjustment to criteria and beta
</commit_message>
<xml_diff>
--- a/Output/Backtest_Table.xlsx
+++ b/Output/Backtest_Table.xlsx
@@ -754,12 +754,12 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>15.91%</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>11.55%</t>
+          <t>11.74%</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>-10.32%</t>
+          <t>-9.74%</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>-9.63%</t>
+          <t>-10.34%</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>14.59%</t>
+          <t>16.31%</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>10.75%</t>
+          <t>10.85%</t>
         </is>
       </c>
       <c r="D10" s="18" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>-11.84%</t>
+          <t>-11.61%</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="G10" s="19" t="inlineStr">
         <is>
-          <t>-10.92%</t>
+          <t>-11.91%</t>
         </is>
       </c>
     </row>
@@ -828,12 +828,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>11.05%</t>
+          <t>12.01%</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>16.17%</t>
+          <t>16.79%</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>21.16%</t>
+          <t>22.64%</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>19.51%</t>
+          <t>21.36%</t>
         </is>
       </c>
     </row>
@@ -865,32 +865,32 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.45</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>-0.49</t>
+          <t>-0.61</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>0.83</t>
+          <t>0.58</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>-0.49</t>
+          <t>-0.68</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>-23.29%</t>
+          <t>-22.04%</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>-39.99%</t>
+          <t>-44.91%</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>-99.81%</t>
+          <t>-99.79%</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="G13" s="22" t="inlineStr">
         <is>
-          <t>-99.70%</t>
+          <t>-99.82%</t>
         </is>
       </c>
     </row>
@@ -946,12 +946,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>2.61</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>-0.66</t>
+          <t>-0.59</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>-0.67</t>
+          <t>-0.65</t>
         </is>
       </c>
     </row>
@@ -983,12 +983,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>0.29</t>
+          <t>0.26</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>-8.68%</t>
+          <t>-10.72%</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>-19.04%</t>
+          <t>-19.64%</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>-20.68%</t>
+          <t>-22.99%</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>-20.20%</t>
+          <t>-23.17%</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>57.9%</t>
+          <t>58.3%</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E18" s="18" t="inlineStr">
         <is>
-          <t>40.7%</t>
+          <t>39.5%</t>
         </is>
       </c>
       <c r="F18" s="18" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>39.5%</t>
         </is>
       </c>
     </row>
@@ -1094,12 +1094,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.13</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>0.64</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.46</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1131,12 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.70</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>2.33</t>
+          <t>2.15</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="F20" s="15" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>2.25</t>
+          <t>2.42</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>9.04</t>
+          <t>9.27</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>4.99</t>
+          <t>4.89</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>-3.41</t>
+          <t>-3.01</t>
         </is>
       </c>
       <c r="F22" s="12" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>-3.45</t>
+          <t>-3.39</t>
         </is>
       </c>
     </row>
@@ -1227,7 +1227,7 @@
       </c>
       <c r="E23" s="18" t="inlineStr">
         <is>
-          <t>0.0007</t>
+          <t>0.0027</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>0.0006</t>
+          <t>0.0008</t>
         </is>
       </c>
     </row>
@@ -1249,12 +1249,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>[11.20%, 17.39%]</t>
+          <t>[12.55%, 19.28%]</t>
         </is>
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>[7.02%, 16.08%]</t>
+          <t>[7.04%, 16.45%]</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>[-16.25%, -4.39%]</t>
+          <t>[-16.08%, -3.39%]</t>
         </is>
       </c>
       <c r="F24" s="21" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G24" s="22" t="inlineStr">
         <is>
-          <t>[-15.09%, -4.16%]</t>
+          <t>[-16.33%, -4.36%]</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>8.27%</t>
+          <t>9.13%</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>6.04%</t>
+          <t>5.71%</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>0.28%</t>
+          <t>1.40%</t>
         </is>
       </c>
       <c r="F26" s="12" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t>0.22%</t>
+          <t>0.15%</t>
         </is>
       </c>
     </row>
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>1.75%</t>
+          <t>1.81%</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>2.42%</t>
+          <t>2.45%</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="E27" s="18" t="inlineStr">
         <is>
-          <t>1.22%</t>
+          <t>1.42%</t>
         </is>
       </c>
       <c r="F27" s="18" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>1.03%</t>
+          <t>1.30%</t>
         </is>
       </c>
     </row>
@@ -1367,12 +1367,12 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>4.71</t>
+          <t>5.03</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.33</t>
         </is>
       </c>
       <c r="D28" s="12" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>0.23</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="F28" s="12" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>0.21</t>
+          <t>0.12</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>0.0124</t>
+          <t>0.0198</t>
         </is>
       </c>
       <c r="D29" s="18" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="E29" s="18" t="inlineStr">
         <is>
-          <t>0.8184</t>
+          <t>0.3247</t>
         </is>
       </c>
       <c r="F29" s="18" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>0.8333</t>
+          <t>0.9064</t>
         </is>
       </c>
     </row>
@@ -1441,12 +1441,12 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>[4.83%, 11.71%]</t>
+          <t>[5.57%, 12.68%]</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>[1.30%, 10.78%]</t>
+          <t>[0.91%, 10.51%]</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>[-2.11%, 2.66%]</t>
+          <t>[-1.39%, 4.18%]</t>
         </is>
       </c>
       <c r="F30" s="12" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>[-1.80%, 2.24%]</t>
+          <t>[-2.39%, 2.70%]</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>0.222</t>
+          <t>0.314</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>0.160</t>
+          <t>0.223</t>
         </is>
       </c>
       <c r="D31" s="18" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>-1.274</t>
+          <t>-1.338</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>-1.183</t>
+          <t>-1.261</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1515,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>7.43</t>
+          <t>10.27</t>
         </is>
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>2.53</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -1530,7 +1530,7 @@
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>-45.54</t>
+          <t>-39.18</t>
         </is>
       </c>
       <c r="F32" s="21" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G32" s="22" t="inlineStr">
         <is>
-          <t>-47.85</t>
+          <t>-36.39</t>
         </is>
       </c>
     </row>

</xml_diff>